<commit_message>
se agregan tareas importantes a corto y mediano plazo, tambien se completo una tarea pendiente
</commit_message>
<xml_diff>
--- a/docs/otros/Estimación Ágil Proyecto Aerolínea.xlsx
+++ b/docs/otros/Estimación Ágil Proyecto Aerolínea.xlsx
@@ -1,17 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{03D72AF1-056A-4C16-9C39-A1D986690E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Estimación Ágil Proyecto Aerolí" sheetId="1" r:id="rId5"/>
+    <sheet name="Estimación Ágil Proyecto Aerolí" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
   <si>
     <t>Talla (T-Shirt)</t>
   </si>
@@ -85,7 +105,7 @@
     <t>2 a 3 semanas</t>
   </si>
   <si>
-    <t>Sistema de Reportes Comerciales y Estadísticas (Ingresos y Clientes frecuentes).</t>
+    <t>Sistema de Reportes Comerciales y Estadisticas (Ingresos y Clientes Frecuentes</t>
   </si>
   <si>
     <t>XXL</t>
@@ -101,26 +121,55 @@
   </si>
   <si>
     <t xml:space="preserve">implementacion del calendario en la seccion de la reserva </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completo </t>
+  </si>
+  <si>
+    <t>2 a 3 dias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">separar el script.js en modulos </t>
+  </si>
+  <si>
+    <t>Validar origen, destino, pasajeros y fechas antes de enviar el formulario</t>
+  </si>
+  <si>
+    <t>Implementar cierre del calendario con tecla ESC</t>
+  </si>
+  <si>
+    <t>Restringir reservas a máximo 1 año en el futuro.</t>
+  </si>
+  <si>
+    <t>Filtrar las ofertas según destino, fechas y tipo de viaje usando lógica en JavaScript</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L </t>
+  </si>
+  <si>
+    <t>Conectar el formulario, almacenamiento, filtrado y renderizado entre páginas.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -131,11 +180,17 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
-    <border/>
+  <borders count="4">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -149,42 +204,76 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -374,24 +463,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="11.5"/>
-    <col customWidth="1" min="2" max="2" width="11.63"/>
-    <col customWidth="1" min="3" max="3" width="16.0"/>
-    <col customWidth="1" min="4" max="4" width="14.88"/>
-    <col customWidth="1" min="5" max="5" width="61.5"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="61.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -407,8 +499,9 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" ht="12.75">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -416,7 +509,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="2">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>7</v>
@@ -424,8 +517,9 @@
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" ht="12.75">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -433,7 +527,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="2">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>11</v>
@@ -441,8 +535,9 @@
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" ht="12.75">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -450,7 +545,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="2">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>15</v>
@@ -458,8 +553,9 @@
       <c r="E4" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="12.75">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -467,7 +563,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="2">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -475,25 +571,27 @@
       <c r="E5" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="24">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="2">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" ht="12.75">
       <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
@@ -501,7 +599,7 @@
         <v>26</v>
       </c>
       <c r="C7" s="2">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>27</v>
@@ -509,8 +607,9 @@
       <c r="E7" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="12.75">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -518,7 +617,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="2">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>11</v>
@@ -526,11 +625,122 @@
       <c r="E8" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="E10" s="3"/>
+      <c r="F8" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="12.75">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="2">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2">
+        <v>8</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" customHeight="1">
+      <c r="E15" s="5"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se añaden nuevas tareas, completamos otras 2 y estan en progreso otras dos
</commit_message>
<xml_diff>
--- a/docs/otros/Estimación Ágil Proyecto Aerolínea.xlsx
+++ b/docs/otros/Estimación Ágil Proyecto Aerolínea.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03D72AF1-056A-4C16-9C39-A1D986690E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E45E44FE-AB34-4A03-8298-A37E53D8DE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="45">
   <si>
     <t>Talla (T-Shirt)</t>
   </si>
@@ -148,13 +148,31 @@
   </si>
   <si>
     <t>Conectar el formulario, almacenamiento, filtrado y renderizado entre páginas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 a 3 dias </t>
+  </si>
+  <si>
+    <t>implementar correctamente con restricciones y conexiones la seccion de el carrito de compras</t>
+  </si>
+  <si>
+    <t>en progreso</t>
+  </si>
+  <si>
+    <t>~7 horas</t>
+  </si>
+  <si>
+    <t>que el calendario no se cierre automaticamente despues de seleccionar una fecha</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -171,6 +189,13 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -236,25 +261,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -473,7 +503,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
@@ -625,7 +655,7 @@
       <c r="E8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -681,9 +711,11 @@
       <c r="E11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F11" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="12.75">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
@@ -699,9 +731,11 @@
       <c r="E12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" customHeight="1">
+      <c r="F12" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="24">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -719,7 +753,7 @@
       </c>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" ht="15.75" customHeight="1">
+    <row r="14" spans="1:6" ht="24">
       <c r="A14" s="2" t="s">
         <v>37</v>
       </c>
@@ -729,16 +763,53 @@
       <c r="C14" s="2">
         <v>8</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" customHeight="1">
-      <c r="E15" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" ht="24">
+      <c r="A15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="5">
+        <v>5</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75" customHeight="1">
+      <c r="A16" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="11">
+        <v>3</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>42</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>